<commit_message>
Dev's India file updates for transportation (1 ccs and 1 indst file too)
</commit_message>
<xml_diff>
--- a/InputData/trans/AVL/Avg Vehicle Lifetime.xlsx
+++ b/InputData/trans/AVL/Avg Vehicle Lifetime.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onewri-my.sharepoint.com/personal/anuj_talwar_wri_org/Documents/EPS/Transport/Input Data/India 3.1.3.5/AVL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\India EPS\InputData\trans\AVL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="143" documentId="13_ncr:1_{683937AB-F5C5-49F8-95B7-31920D8FD88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24D542DD-80FA-4FD1-9BCE-1979711DF904}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{427B8E0F-9937-4961-A5AE-03C7019D44DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="19188" windowHeight="11208" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="9" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="73">
   <si>
     <t>AVL Avg Vehicle Lifetime</t>
   </si>
@@ -257,6 +257,9 @@
   </si>
   <si>
     <t>rail</t>
+  </si>
+  <si>
+    <t>&lt;using US data here</t>
   </si>
   <si>
     <t>motorbikes</t>
@@ -286,7 +289,7 @@
     <numFmt numFmtId="178" formatCode="0.0_ ;\-0.0\ "/>
     <numFmt numFmtId="179" formatCode="0.0%;\ \(0.0%\);\ \-"/>
   </numFmts>
-  <fonts count="105">
+  <fonts count="106">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -961,8 +964,14 @@
       <family val="1"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="66">
+  <fills count="65">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1163,12 +1172,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2410,6 +2413,7 @@
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="29" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="57" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="57" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="57" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="57" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2418,17 +2422,16 @@
     <xf numFmtId="0" fontId="57" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="57" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="57" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="57" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="57" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="57" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="57" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="57" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="57" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="58" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="58" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="58" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="58" fillId="49" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="58" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="58" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="58" fillId="50" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="58" fillId="51" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="58" fillId="52" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="29" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="4" fontId="59" fillId="0" borderId="29" applyFill="0">
@@ -2440,17 +2443,17 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="60" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="0" fontId="61" fillId="53" borderId="30" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="53" borderId="30" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="53" borderId="30" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="52" borderId="30" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="52" borderId="30" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="52" borderId="30" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="62" fillId="0" borderId="31" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="63" fillId="54" borderId="32" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="63" fillId="53" borderId="32" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="58" fillId="54" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="58" fillId="55" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="58" fillId="56" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="58" fillId="49" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="58" fillId="50" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="58" fillId="57" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="58" fillId="50" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="58" fillId="51" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="58" fillId="58" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="64" fillId="0" borderId="18">
@@ -2483,7 +2486,7 @@
     <xf numFmtId="0" fontId="70" fillId="0" borderId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="38" fontId="71" fillId="59" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="38" fontId="71" fillId="58" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="27" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2500,9 +2503,9 @@
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="10" fontId="71" fillId="60" borderId="28" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="10" fontId="71" fillId="60" borderId="28" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="10" fontId="71" fillId="60" borderId="28" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="10" fontId="71" fillId="59" borderId="28" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="10" fontId="71" fillId="59" borderId="28" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="10" fontId="71" fillId="59" borderId="28" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="176" fontId="73" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyBorder="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2510,7 +2513,7 @@
     <xf numFmtId="167" fontId="75" fillId="0" borderId="26">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="76" fillId="61" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="60" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="37" fontId="77" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="29" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
@@ -2529,9 +2532,9 @@
     <xf numFmtId="0" fontId="79" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="80" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="62" borderId="33" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="62" borderId="33" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="62" borderId="33" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="29" fillId="61" borderId="33" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="29" fillId="61" borderId="33" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="29" fillId="61" borderId="33" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="34"/>
@@ -2576,7 +2579,7 @@
     <xf numFmtId="0" fontId="85" fillId="0" borderId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="86" fillId="63" borderId="0" applyNumberFormat="0" applyFill="0">
+    <xf numFmtId="0" fontId="86" fillId="62" borderId="0" applyNumberFormat="0" applyFill="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="40" fontId="87" fillId="0" borderId="0" applyBorder="0">
@@ -2602,8 +2605,8 @@
     <xf numFmtId="0" fontId="97" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="97" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="97" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="98" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="99" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="98" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="99" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="171" fontId="31" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2630,7 +2633,7 @@
     <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="170" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="100" fillId="64" borderId="0"/>
+    <xf numFmtId="0" fontId="100" fillId="63" borderId="0"/>
     <xf numFmtId="167" fontId="101" fillId="35" borderId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -2749,9 +2752,9 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="53" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="53" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="53" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="52" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="52" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="52" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="64" fillId="0" borderId="41">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -2764,12 +2767,12 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="39">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="71" fillId="60" borderId="40" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="10" fontId="71" fillId="60" borderId="40" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="10" fontId="71" fillId="60" borderId="40" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="62" borderId="44" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="62" borderId="44" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="62" borderId="44" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="10" fontId="71" fillId="59" borderId="40" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="10" fontId="71" fillId="59" borderId="40" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="10" fontId="71" fillId="59" borderId="40" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="29" fillId="61" borderId="44" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="29" fillId="61" borderId="44" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="29" fillId="61" borderId="44" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="45"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="45"/>
     <xf numFmtId="0" fontId="85" fillId="0" borderId="40">
@@ -2814,7 +2817,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="36" borderId="0" xfId="64" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="38" fillId="38" borderId="0" xfId="64" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="38" fillId="37" borderId="0" xfId="64" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="169" fontId="36" fillId="36" borderId="25" xfId="573" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -2839,12 +2842,11 @@
     <xf numFmtId="173" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="102" fillId="65" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="102" fillId="64" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="103" fillId="38" borderId="0" xfId="64" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="103" fillId="37" borderId="0" xfId="64" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="103" fillId="36" borderId="0" xfId="64" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="34" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -2923,6 +2925,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="702"/>
+    <xf numFmtId="0" fontId="105" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="703">
     <cellStyle name="20% - Accent1" xfId="33" builtinId="30" customBuiltin="1"/>
@@ -3122,343 +3125,343 @@
     <cellStyle name="Hed Side Regular" xfId="58" xr:uid="{00000000-0005-0000-0000-0000C2000000}"/>
     <cellStyle name="Hed Top" xfId="57" xr:uid="{00000000-0005-0000-0000-0000C3000000}"/>
     <cellStyle name="Hyperlink" xfId="702" builtinId="8"/>
+    <cellStyle name="Hyperlink 10" xfId="280" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C5000000}"/>
     <cellStyle name="Hyperlink 10" xfId="125" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C4000000}"/>
-    <cellStyle name="Hyperlink 10" xfId="280" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C5000000}"/>
     <cellStyle name="Hyperlink 10" xfId="615" xr:uid="{00000000-0005-0000-0000-0000C6000000}"/>
+    <cellStyle name="Hyperlink 100" xfId="330" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C8000000}"/>
     <cellStyle name="Hyperlink 100" xfId="215" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C7000000}"/>
-    <cellStyle name="Hyperlink 100" xfId="330" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C8000000}"/>
     <cellStyle name="Hyperlink 100" xfId="665" xr:uid="{00000000-0005-0000-0000-0000C9000000}"/>
+    <cellStyle name="Hyperlink 101" xfId="331" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CB000000}"/>
     <cellStyle name="Hyperlink 101" xfId="216" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CA000000}"/>
-    <cellStyle name="Hyperlink 101" xfId="331" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CB000000}"/>
     <cellStyle name="Hyperlink 101" xfId="666" xr:uid="{00000000-0005-0000-0000-0000CC000000}"/>
+    <cellStyle name="Hyperlink 102" xfId="332" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CE000000}"/>
     <cellStyle name="Hyperlink 102" xfId="217" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CD000000}"/>
-    <cellStyle name="Hyperlink 102" xfId="332" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CE000000}"/>
     <cellStyle name="Hyperlink 102" xfId="667" xr:uid="{00000000-0005-0000-0000-0000CF000000}"/>
+    <cellStyle name="Hyperlink 103" xfId="333" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D1000000}"/>
     <cellStyle name="Hyperlink 103" xfId="218" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D0000000}"/>
-    <cellStyle name="Hyperlink 103" xfId="333" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D1000000}"/>
     <cellStyle name="Hyperlink 103" xfId="668" xr:uid="{00000000-0005-0000-0000-0000D2000000}"/>
+    <cellStyle name="Hyperlink 104" xfId="334" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D4000000}"/>
     <cellStyle name="Hyperlink 104" xfId="219" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D3000000}"/>
-    <cellStyle name="Hyperlink 104" xfId="334" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D4000000}"/>
     <cellStyle name="Hyperlink 104" xfId="669" xr:uid="{00000000-0005-0000-0000-0000D5000000}"/>
+    <cellStyle name="Hyperlink 105" xfId="335" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D7000000}"/>
     <cellStyle name="Hyperlink 105" xfId="220" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D6000000}"/>
-    <cellStyle name="Hyperlink 105" xfId="335" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D7000000}"/>
     <cellStyle name="Hyperlink 105" xfId="670" xr:uid="{00000000-0005-0000-0000-0000D8000000}"/>
+    <cellStyle name="Hyperlink 106" xfId="336" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DA000000}"/>
     <cellStyle name="Hyperlink 106" xfId="221" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D9000000}"/>
-    <cellStyle name="Hyperlink 106" xfId="336" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DA000000}"/>
     <cellStyle name="Hyperlink 106" xfId="671" xr:uid="{00000000-0005-0000-0000-0000DB000000}"/>
+    <cellStyle name="Hyperlink 107" xfId="337" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DD000000}"/>
     <cellStyle name="Hyperlink 107" xfId="222" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DC000000}"/>
-    <cellStyle name="Hyperlink 107" xfId="337" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DD000000}"/>
     <cellStyle name="Hyperlink 107" xfId="672" xr:uid="{00000000-0005-0000-0000-0000DE000000}"/>
+    <cellStyle name="Hyperlink 108" xfId="338" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E0000000}"/>
     <cellStyle name="Hyperlink 108" xfId="223" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DF000000}"/>
-    <cellStyle name="Hyperlink 108" xfId="338" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E0000000}"/>
     <cellStyle name="Hyperlink 108" xfId="673" xr:uid="{00000000-0005-0000-0000-0000E1000000}"/>
+    <cellStyle name="Hyperlink 109" xfId="339" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E3000000}"/>
     <cellStyle name="Hyperlink 109" xfId="224" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E2000000}"/>
-    <cellStyle name="Hyperlink 109" xfId="339" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E3000000}"/>
     <cellStyle name="Hyperlink 109" xfId="674" xr:uid="{00000000-0005-0000-0000-0000E4000000}"/>
+    <cellStyle name="Hyperlink 11" xfId="279" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E6000000}"/>
     <cellStyle name="Hyperlink 11" xfId="126" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E5000000}"/>
-    <cellStyle name="Hyperlink 11" xfId="279" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E6000000}"/>
     <cellStyle name="Hyperlink 11" xfId="614" xr:uid="{00000000-0005-0000-0000-0000E7000000}"/>
+    <cellStyle name="Hyperlink 110" xfId="340" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E9000000}"/>
     <cellStyle name="Hyperlink 110" xfId="225" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E8000000}"/>
-    <cellStyle name="Hyperlink 110" xfId="340" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E9000000}"/>
     <cellStyle name="Hyperlink 110" xfId="675" xr:uid="{00000000-0005-0000-0000-0000EA000000}"/>
+    <cellStyle name="Hyperlink 111" xfId="341" hidden="1" xr:uid="{00000000-0005-0000-0000-0000EC000000}"/>
     <cellStyle name="Hyperlink 111" xfId="226" hidden="1" xr:uid="{00000000-0005-0000-0000-0000EB000000}"/>
-    <cellStyle name="Hyperlink 111" xfId="341" hidden="1" xr:uid="{00000000-0005-0000-0000-0000EC000000}"/>
     <cellStyle name="Hyperlink 111" xfId="676" xr:uid="{00000000-0005-0000-0000-0000ED000000}"/>
     <cellStyle name="Hyperlink 112" xfId="555" xr:uid="{00000000-0005-0000-0000-0000EE000000}"/>
     <cellStyle name="Hyperlink 113" xfId="115" xr:uid="{00000000-0005-0000-0000-0000EF000000}"/>
+    <cellStyle name="Hyperlink 12" xfId="278" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F1000000}"/>
     <cellStyle name="Hyperlink 12" xfId="127" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F0000000}"/>
-    <cellStyle name="Hyperlink 12" xfId="278" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F1000000}"/>
     <cellStyle name="Hyperlink 12" xfId="613" xr:uid="{00000000-0005-0000-0000-0000F2000000}"/>
+    <cellStyle name="Hyperlink 13" xfId="277" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F4000000}"/>
     <cellStyle name="Hyperlink 13" xfId="128" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F3000000}"/>
-    <cellStyle name="Hyperlink 13" xfId="277" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F4000000}"/>
     <cellStyle name="Hyperlink 13" xfId="612" xr:uid="{00000000-0005-0000-0000-0000F5000000}"/>
+    <cellStyle name="Hyperlink 14" xfId="276" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F7000000}"/>
     <cellStyle name="Hyperlink 14" xfId="129" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F6000000}"/>
-    <cellStyle name="Hyperlink 14" xfId="276" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F7000000}"/>
     <cellStyle name="Hyperlink 14" xfId="68" xr:uid="{00000000-0005-0000-0000-0000F8000000}"/>
+    <cellStyle name="Hyperlink 15" xfId="275" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FA000000}"/>
     <cellStyle name="Hyperlink 15" xfId="130" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F9000000}"/>
-    <cellStyle name="Hyperlink 15" xfId="275" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FA000000}"/>
     <cellStyle name="Hyperlink 15" xfId="69" xr:uid="{00000000-0005-0000-0000-0000FB000000}"/>
+    <cellStyle name="Hyperlink 16" xfId="274" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FD000000}"/>
     <cellStyle name="Hyperlink 16" xfId="131" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FC000000}"/>
-    <cellStyle name="Hyperlink 16" xfId="274" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FD000000}"/>
     <cellStyle name="Hyperlink 16" xfId="70" xr:uid="{00000000-0005-0000-0000-0000FE000000}"/>
+    <cellStyle name="Hyperlink 17" xfId="273" hidden="1" xr:uid="{00000000-0005-0000-0000-000000010000}"/>
     <cellStyle name="Hyperlink 17" xfId="132" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FF000000}"/>
-    <cellStyle name="Hyperlink 17" xfId="273" hidden="1" xr:uid="{00000000-0005-0000-0000-000000010000}"/>
     <cellStyle name="Hyperlink 17" xfId="71" xr:uid="{00000000-0005-0000-0000-000001010000}"/>
+    <cellStyle name="Hyperlink 18" xfId="272" hidden="1" xr:uid="{00000000-0005-0000-0000-000003010000}"/>
     <cellStyle name="Hyperlink 18" xfId="133" hidden="1" xr:uid="{00000000-0005-0000-0000-000002010000}"/>
-    <cellStyle name="Hyperlink 18" xfId="272" hidden="1" xr:uid="{00000000-0005-0000-0000-000003010000}"/>
     <cellStyle name="Hyperlink 18" xfId="72" xr:uid="{00000000-0005-0000-0000-000004010000}"/>
+    <cellStyle name="Hyperlink 19" xfId="271" hidden="1" xr:uid="{00000000-0005-0000-0000-000006010000}"/>
     <cellStyle name="Hyperlink 19" xfId="134" hidden="1" xr:uid="{00000000-0005-0000-0000-000005010000}"/>
-    <cellStyle name="Hyperlink 19" xfId="271" hidden="1" xr:uid="{00000000-0005-0000-0000-000006010000}"/>
     <cellStyle name="Hyperlink 19" xfId="73" xr:uid="{00000000-0005-0000-0000-000007010000}"/>
     <cellStyle name="Hyperlink 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000008010000}"/>
     <cellStyle name="Hyperlink 2 2" xfId="480" xr:uid="{00000000-0005-0000-0000-000009010000}"/>
+    <cellStyle name="Hyperlink 2 3" xfId="113" hidden="1" xr:uid="{00000000-0005-0000-0000-00000E010000}"/>
+    <cellStyle name="Hyperlink 2 3" xfId="623" hidden="1" xr:uid="{00000000-0005-0000-0000-00000F010000}"/>
+    <cellStyle name="Hyperlink 2 3" xfId="288" hidden="1" xr:uid="{00000000-0005-0000-0000-00000C010000}"/>
+    <cellStyle name="Hyperlink 2 3" xfId="342" hidden="1" xr:uid="{00000000-0005-0000-0000-00000D010000}"/>
     <cellStyle name="Hyperlink 2 3" xfId="228" hidden="1" xr:uid="{00000000-0005-0000-0000-00000B010000}"/>
     <cellStyle name="Hyperlink 2 3" xfId="116" hidden="1" xr:uid="{00000000-0005-0000-0000-00000A010000}"/>
-    <cellStyle name="Hyperlink 2 3" xfId="288" hidden="1" xr:uid="{00000000-0005-0000-0000-00000C010000}"/>
-    <cellStyle name="Hyperlink 2 3" xfId="342" hidden="1" xr:uid="{00000000-0005-0000-0000-00000D010000}"/>
-    <cellStyle name="Hyperlink 2 3" xfId="623" hidden="1" xr:uid="{00000000-0005-0000-0000-00000F010000}"/>
-    <cellStyle name="Hyperlink 2 3" xfId="113" hidden="1" xr:uid="{00000000-0005-0000-0000-00000E010000}"/>
     <cellStyle name="Hyperlink 2 3" xfId="677" xr:uid="{00000000-0005-0000-0000-000010010000}"/>
+    <cellStyle name="Hyperlink 20" xfId="270" hidden="1" xr:uid="{00000000-0005-0000-0000-000012010000}"/>
     <cellStyle name="Hyperlink 20" xfId="135" hidden="1" xr:uid="{00000000-0005-0000-0000-000011010000}"/>
-    <cellStyle name="Hyperlink 20" xfId="270" hidden="1" xr:uid="{00000000-0005-0000-0000-000012010000}"/>
     <cellStyle name="Hyperlink 20" xfId="74" xr:uid="{00000000-0005-0000-0000-000013010000}"/>
+    <cellStyle name="Hyperlink 21" xfId="269" hidden="1" xr:uid="{00000000-0005-0000-0000-000015010000}"/>
     <cellStyle name="Hyperlink 21" xfId="136" hidden="1" xr:uid="{00000000-0005-0000-0000-000014010000}"/>
-    <cellStyle name="Hyperlink 21" xfId="269" hidden="1" xr:uid="{00000000-0005-0000-0000-000015010000}"/>
     <cellStyle name="Hyperlink 21" xfId="75" xr:uid="{00000000-0005-0000-0000-000016010000}"/>
+    <cellStyle name="Hyperlink 22" xfId="268" hidden="1" xr:uid="{00000000-0005-0000-0000-000018010000}"/>
     <cellStyle name="Hyperlink 22" xfId="137" hidden="1" xr:uid="{00000000-0005-0000-0000-000017010000}"/>
-    <cellStyle name="Hyperlink 22" xfId="268" hidden="1" xr:uid="{00000000-0005-0000-0000-000018010000}"/>
     <cellStyle name="Hyperlink 22" xfId="76" xr:uid="{00000000-0005-0000-0000-000019010000}"/>
+    <cellStyle name="Hyperlink 23" xfId="267" hidden="1" xr:uid="{00000000-0005-0000-0000-00001B010000}"/>
     <cellStyle name="Hyperlink 23" xfId="138" hidden="1" xr:uid="{00000000-0005-0000-0000-00001A010000}"/>
-    <cellStyle name="Hyperlink 23" xfId="267" hidden="1" xr:uid="{00000000-0005-0000-0000-00001B010000}"/>
     <cellStyle name="Hyperlink 23" xfId="77" xr:uid="{00000000-0005-0000-0000-00001C010000}"/>
+    <cellStyle name="Hyperlink 24" xfId="266" hidden="1" xr:uid="{00000000-0005-0000-0000-00001E010000}"/>
     <cellStyle name="Hyperlink 24" xfId="139" hidden="1" xr:uid="{00000000-0005-0000-0000-00001D010000}"/>
-    <cellStyle name="Hyperlink 24" xfId="266" hidden="1" xr:uid="{00000000-0005-0000-0000-00001E010000}"/>
     <cellStyle name="Hyperlink 24" xfId="78" xr:uid="{00000000-0005-0000-0000-00001F010000}"/>
+    <cellStyle name="Hyperlink 25" xfId="265" hidden="1" xr:uid="{00000000-0005-0000-0000-000021010000}"/>
     <cellStyle name="Hyperlink 25" xfId="140" hidden="1" xr:uid="{00000000-0005-0000-0000-000020010000}"/>
-    <cellStyle name="Hyperlink 25" xfId="265" hidden="1" xr:uid="{00000000-0005-0000-0000-000021010000}"/>
     <cellStyle name="Hyperlink 25" xfId="79" xr:uid="{00000000-0005-0000-0000-000022010000}"/>
+    <cellStyle name="Hyperlink 26" xfId="264" hidden="1" xr:uid="{00000000-0005-0000-0000-000024010000}"/>
     <cellStyle name="Hyperlink 26" xfId="141" hidden="1" xr:uid="{00000000-0005-0000-0000-000023010000}"/>
-    <cellStyle name="Hyperlink 26" xfId="264" hidden="1" xr:uid="{00000000-0005-0000-0000-000024010000}"/>
     <cellStyle name="Hyperlink 26" xfId="80" xr:uid="{00000000-0005-0000-0000-000025010000}"/>
+    <cellStyle name="Hyperlink 27" xfId="263" hidden="1" xr:uid="{00000000-0005-0000-0000-000027010000}"/>
     <cellStyle name="Hyperlink 27" xfId="142" hidden="1" xr:uid="{00000000-0005-0000-0000-000026010000}"/>
-    <cellStyle name="Hyperlink 27" xfId="263" hidden="1" xr:uid="{00000000-0005-0000-0000-000027010000}"/>
     <cellStyle name="Hyperlink 27" xfId="81" xr:uid="{00000000-0005-0000-0000-000028010000}"/>
+    <cellStyle name="Hyperlink 28" xfId="262" hidden="1" xr:uid="{00000000-0005-0000-0000-00002A010000}"/>
     <cellStyle name="Hyperlink 28" xfId="143" hidden="1" xr:uid="{00000000-0005-0000-0000-000029010000}"/>
-    <cellStyle name="Hyperlink 28" xfId="262" hidden="1" xr:uid="{00000000-0005-0000-0000-00002A010000}"/>
     <cellStyle name="Hyperlink 28" xfId="82" xr:uid="{00000000-0005-0000-0000-00002B010000}"/>
+    <cellStyle name="Hyperlink 29" xfId="261" hidden="1" xr:uid="{00000000-0005-0000-0000-00002D010000}"/>
     <cellStyle name="Hyperlink 29" xfId="144" hidden="1" xr:uid="{00000000-0005-0000-0000-00002C010000}"/>
-    <cellStyle name="Hyperlink 29" xfId="261" hidden="1" xr:uid="{00000000-0005-0000-0000-00002D010000}"/>
     <cellStyle name="Hyperlink 29" xfId="83" xr:uid="{00000000-0005-0000-0000-00002E010000}"/>
+    <cellStyle name="Hyperlink 3" xfId="287" hidden="1" xr:uid="{00000000-0005-0000-0000-000030010000}"/>
     <cellStyle name="Hyperlink 3" xfId="118" hidden="1" xr:uid="{00000000-0005-0000-0000-00002F010000}"/>
-    <cellStyle name="Hyperlink 3" xfId="287" hidden="1" xr:uid="{00000000-0005-0000-0000-000030010000}"/>
     <cellStyle name="Hyperlink 3" xfId="622" xr:uid="{00000000-0005-0000-0000-000031010000}"/>
+    <cellStyle name="Hyperlink 30" xfId="260" hidden="1" xr:uid="{00000000-0005-0000-0000-000033010000}"/>
     <cellStyle name="Hyperlink 30" xfId="145" hidden="1" xr:uid="{00000000-0005-0000-0000-000032010000}"/>
-    <cellStyle name="Hyperlink 30" xfId="260" hidden="1" xr:uid="{00000000-0005-0000-0000-000033010000}"/>
     <cellStyle name="Hyperlink 30" xfId="84" xr:uid="{00000000-0005-0000-0000-000034010000}"/>
+    <cellStyle name="Hyperlink 31" xfId="259" hidden="1" xr:uid="{00000000-0005-0000-0000-000036010000}"/>
     <cellStyle name="Hyperlink 31" xfId="146" hidden="1" xr:uid="{00000000-0005-0000-0000-000035010000}"/>
-    <cellStyle name="Hyperlink 31" xfId="259" hidden="1" xr:uid="{00000000-0005-0000-0000-000036010000}"/>
     <cellStyle name="Hyperlink 31" xfId="85" xr:uid="{00000000-0005-0000-0000-000037010000}"/>
+    <cellStyle name="Hyperlink 32" xfId="258" hidden="1" xr:uid="{00000000-0005-0000-0000-000039010000}"/>
     <cellStyle name="Hyperlink 32" xfId="147" hidden="1" xr:uid="{00000000-0005-0000-0000-000038010000}"/>
-    <cellStyle name="Hyperlink 32" xfId="258" hidden="1" xr:uid="{00000000-0005-0000-0000-000039010000}"/>
     <cellStyle name="Hyperlink 32" xfId="86" xr:uid="{00000000-0005-0000-0000-00003A010000}"/>
+    <cellStyle name="Hyperlink 33" xfId="257" hidden="1" xr:uid="{00000000-0005-0000-0000-00003C010000}"/>
     <cellStyle name="Hyperlink 33" xfId="148" hidden="1" xr:uid="{00000000-0005-0000-0000-00003B010000}"/>
-    <cellStyle name="Hyperlink 33" xfId="257" hidden="1" xr:uid="{00000000-0005-0000-0000-00003C010000}"/>
     <cellStyle name="Hyperlink 33" xfId="87" xr:uid="{00000000-0005-0000-0000-00003D010000}"/>
+    <cellStyle name="Hyperlink 34" xfId="256" hidden="1" xr:uid="{00000000-0005-0000-0000-00003F010000}"/>
     <cellStyle name="Hyperlink 34" xfId="149" hidden="1" xr:uid="{00000000-0005-0000-0000-00003E010000}"/>
-    <cellStyle name="Hyperlink 34" xfId="256" hidden="1" xr:uid="{00000000-0005-0000-0000-00003F010000}"/>
     <cellStyle name="Hyperlink 34" xfId="88" xr:uid="{00000000-0005-0000-0000-000040010000}"/>
+    <cellStyle name="Hyperlink 35" xfId="255" hidden="1" xr:uid="{00000000-0005-0000-0000-000042010000}"/>
     <cellStyle name="Hyperlink 35" xfId="150" hidden="1" xr:uid="{00000000-0005-0000-0000-000041010000}"/>
-    <cellStyle name="Hyperlink 35" xfId="255" hidden="1" xr:uid="{00000000-0005-0000-0000-000042010000}"/>
     <cellStyle name="Hyperlink 35" xfId="89" xr:uid="{00000000-0005-0000-0000-000043010000}"/>
+    <cellStyle name="Hyperlink 36" xfId="254" hidden="1" xr:uid="{00000000-0005-0000-0000-000045010000}"/>
     <cellStyle name="Hyperlink 36" xfId="151" hidden="1" xr:uid="{00000000-0005-0000-0000-000044010000}"/>
-    <cellStyle name="Hyperlink 36" xfId="254" hidden="1" xr:uid="{00000000-0005-0000-0000-000045010000}"/>
     <cellStyle name="Hyperlink 36" xfId="90" xr:uid="{00000000-0005-0000-0000-000046010000}"/>
+    <cellStyle name="Hyperlink 37" xfId="253" hidden="1" xr:uid="{00000000-0005-0000-0000-000048010000}"/>
     <cellStyle name="Hyperlink 37" xfId="152" hidden="1" xr:uid="{00000000-0005-0000-0000-000047010000}"/>
-    <cellStyle name="Hyperlink 37" xfId="253" hidden="1" xr:uid="{00000000-0005-0000-0000-000048010000}"/>
     <cellStyle name="Hyperlink 37" xfId="91" xr:uid="{00000000-0005-0000-0000-000049010000}"/>
+    <cellStyle name="Hyperlink 38" xfId="252" hidden="1" xr:uid="{00000000-0005-0000-0000-00004B010000}"/>
     <cellStyle name="Hyperlink 38" xfId="153" hidden="1" xr:uid="{00000000-0005-0000-0000-00004A010000}"/>
-    <cellStyle name="Hyperlink 38" xfId="252" hidden="1" xr:uid="{00000000-0005-0000-0000-00004B010000}"/>
     <cellStyle name="Hyperlink 38" xfId="92" xr:uid="{00000000-0005-0000-0000-00004C010000}"/>
+    <cellStyle name="Hyperlink 39" xfId="251" hidden="1" xr:uid="{00000000-0005-0000-0000-00004E010000}"/>
     <cellStyle name="Hyperlink 39" xfId="154" hidden="1" xr:uid="{00000000-0005-0000-0000-00004D010000}"/>
-    <cellStyle name="Hyperlink 39" xfId="251" hidden="1" xr:uid="{00000000-0005-0000-0000-00004E010000}"/>
     <cellStyle name="Hyperlink 39" xfId="93" xr:uid="{00000000-0005-0000-0000-00004F010000}"/>
+    <cellStyle name="Hyperlink 4" xfId="286" hidden="1" xr:uid="{00000000-0005-0000-0000-000051010000}"/>
     <cellStyle name="Hyperlink 4" xfId="119" hidden="1" xr:uid="{00000000-0005-0000-0000-000050010000}"/>
-    <cellStyle name="Hyperlink 4" xfId="286" hidden="1" xr:uid="{00000000-0005-0000-0000-000051010000}"/>
     <cellStyle name="Hyperlink 4" xfId="621" xr:uid="{00000000-0005-0000-0000-000052010000}"/>
+    <cellStyle name="Hyperlink 40" xfId="250" hidden="1" xr:uid="{00000000-0005-0000-0000-000054010000}"/>
     <cellStyle name="Hyperlink 40" xfId="155" hidden="1" xr:uid="{00000000-0005-0000-0000-000053010000}"/>
-    <cellStyle name="Hyperlink 40" xfId="250" hidden="1" xr:uid="{00000000-0005-0000-0000-000054010000}"/>
     <cellStyle name="Hyperlink 40" xfId="94" xr:uid="{00000000-0005-0000-0000-000055010000}"/>
+    <cellStyle name="Hyperlink 41" xfId="249" hidden="1" xr:uid="{00000000-0005-0000-0000-000057010000}"/>
     <cellStyle name="Hyperlink 41" xfId="156" hidden="1" xr:uid="{00000000-0005-0000-0000-000056010000}"/>
-    <cellStyle name="Hyperlink 41" xfId="249" hidden="1" xr:uid="{00000000-0005-0000-0000-000057010000}"/>
     <cellStyle name="Hyperlink 41" xfId="95" xr:uid="{00000000-0005-0000-0000-000058010000}"/>
+    <cellStyle name="Hyperlink 42" xfId="248" hidden="1" xr:uid="{00000000-0005-0000-0000-00005A010000}"/>
     <cellStyle name="Hyperlink 42" xfId="157" hidden="1" xr:uid="{00000000-0005-0000-0000-000059010000}"/>
-    <cellStyle name="Hyperlink 42" xfId="248" hidden="1" xr:uid="{00000000-0005-0000-0000-00005A010000}"/>
     <cellStyle name="Hyperlink 42" xfId="96" xr:uid="{00000000-0005-0000-0000-00005B010000}"/>
+    <cellStyle name="Hyperlink 43" xfId="247" hidden="1" xr:uid="{00000000-0005-0000-0000-00005D010000}"/>
     <cellStyle name="Hyperlink 43" xfId="158" hidden="1" xr:uid="{00000000-0005-0000-0000-00005C010000}"/>
-    <cellStyle name="Hyperlink 43" xfId="247" hidden="1" xr:uid="{00000000-0005-0000-0000-00005D010000}"/>
     <cellStyle name="Hyperlink 43" xfId="97" xr:uid="{00000000-0005-0000-0000-00005E010000}"/>
+    <cellStyle name="Hyperlink 44" xfId="246" hidden="1" xr:uid="{00000000-0005-0000-0000-000060010000}"/>
     <cellStyle name="Hyperlink 44" xfId="159" hidden="1" xr:uid="{00000000-0005-0000-0000-00005F010000}"/>
-    <cellStyle name="Hyperlink 44" xfId="246" hidden="1" xr:uid="{00000000-0005-0000-0000-000060010000}"/>
     <cellStyle name="Hyperlink 44" xfId="98" xr:uid="{00000000-0005-0000-0000-000061010000}"/>
+    <cellStyle name="Hyperlink 45" xfId="245" hidden="1" xr:uid="{00000000-0005-0000-0000-000063010000}"/>
     <cellStyle name="Hyperlink 45" xfId="160" hidden="1" xr:uid="{00000000-0005-0000-0000-000062010000}"/>
-    <cellStyle name="Hyperlink 45" xfId="245" hidden="1" xr:uid="{00000000-0005-0000-0000-000063010000}"/>
     <cellStyle name="Hyperlink 45" xfId="99" xr:uid="{00000000-0005-0000-0000-000064010000}"/>
+    <cellStyle name="Hyperlink 46" xfId="244" hidden="1" xr:uid="{00000000-0005-0000-0000-000066010000}"/>
     <cellStyle name="Hyperlink 46" xfId="161" hidden="1" xr:uid="{00000000-0005-0000-0000-000065010000}"/>
-    <cellStyle name="Hyperlink 46" xfId="244" hidden="1" xr:uid="{00000000-0005-0000-0000-000066010000}"/>
     <cellStyle name="Hyperlink 46" xfId="100" xr:uid="{00000000-0005-0000-0000-000067010000}"/>
+    <cellStyle name="Hyperlink 47" xfId="243" hidden="1" xr:uid="{00000000-0005-0000-0000-000069010000}"/>
     <cellStyle name="Hyperlink 47" xfId="162" hidden="1" xr:uid="{00000000-0005-0000-0000-000068010000}"/>
-    <cellStyle name="Hyperlink 47" xfId="243" hidden="1" xr:uid="{00000000-0005-0000-0000-000069010000}"/>
     <cellStyle name="Hyperlink 47" xfId="101" xr:uid="{00000000-0005-0000-0000-00006A010000}"/>
+    <cellStyle name="Hyperlink 48" xfId="242" hidden="1" xr:uid="{00000000-0005-0000-0000-00006C010000}"/>
     <cellStyle name="Hyperlink 48" xfId="163" hidden="1" xr:uid="{00000000-0005-0000-0000-00006B010000}"/>
-    <cellStyle name="Hyperlink 48" xfId="242" hidden="1" xr:uid="{00000000-0005-0000-0000-00006C010000}"/>
     <cellStyle name="Hyperlink 48" xfId="102" xr:uid="{00000000-0005-0000-0000-00006D010000}"/>
+    <cellStyle name="Hyperlink 49" xfId="241" hidden="1" xr:uid="{00000000-0005-0000-0000-00006F010000}"/>
     <cellStyle name="Hyperlink 49" xfId="164" hidden="1" xr:uid="{00000000-0005-0000-0000-00006E010000}"/>
-    <cellStyle name="Hyperlink 49" xfId="241" hidden="1" xr:uid="{00000000-0005-0000-0000-00006F010000}"/>
     <cellStyle name="Hyperlink 49" xfId="103" xr:uid="{00000000-0005-0000-0000-000070010000}"/>
+    <cellStyle name="Hyperlink 5" xfId="285" hidden="1" xr:uid="{00000000-0005-0000-0000-000072010000}"/>
     <cellStyle name="Hyperlink 5" xfId="120" hidden="1" xr:uid="{00000000-0005-0000-0000-000071010000}"/>
-    <cellStyle name="Hyperlink 5" xfId="285" hidden="1" xr:uid="{00000000-0005-0000-0000-000072010000}"/>
     <cellStyle name="Hyperlink 5" xfId="620" xr:uid="{00000000-0005-0000-0000-000073010000}"/>
+    <cellStyle name="Hyperlink 50" xfId="240" hidden="1" xr:uid="{00000000-0005-0000-0000-000075010000}"/>
     <cellStyle name="Hyperlink 50" xfId="165" hidden="1" xr:uid="{00000000-0005-0000-0000-000074010000}"/>
-    <cellStyle name="Hyperlink 50" xfId="240" hidden="1" xr:uid="{00000000-0005-0000-0000-000075010000}"/>
     <cellStyle name="Hyperlink 50" xfId="104" xr:uid="{00000000-0005-0000-0000-000076010000}"/>
+    <cellStyle name="Hyperlink 51" xfId="239" hidden="1" xr:uid="{00000000-0005-0000-0000-000078010000}"/>
     <cellStyle name="Hyperlink 51" xfId="166" hidden="1" xr:uid="{00000000-0005-0000-0000-000077010000}"/>
-    <cellStyle name="Hyperlink 51" xfId="239" hidden="1" xr:uid="{00000000-0005-0000-0000-000078010000}"/>
     <cellStyle name="Hyperlink 51" xfId="105" xr:uid="{00000000-0005-0000-0000-000079010000}"/>
+    <cellStyle name="Hyperlink 52" xfId="238" hidden="1" xr:uid="{00000000-0005-0000-0000-00007B010000}"/>
     <cellStyle name="Hyperlink 52" xfId="167" hidden="1" xr:uid="{00000000-0005-0000-0000-00007A010000}"/>
-    <cellStyle name="Hyperlink 52" xfId="238" hidden="1" xr:uid="{00000000-0005-0000-0000-00007B010000}"/>
     <cellStyle name="Hyperlink 52" xfId="106" xr:uid="{00000000-0005-0000-0000-00007C010000}"/>
+    <cellStyle name="Hyperlink 53" xfId="237" hidden="1" xr:uid="{00000000-0005-0000-0000-00007E010000}"/>
     <cellStyle name="Hyperlink 53" xfId="168" hidden="1" xr:uid="{00000000-0005-0000-0000-00007D010000}"/>
-    <cellStyle name="Hyperlink 53" xfId="237" hidden="1" xr:uid="{00000000-0005-0000-0000-00007E010000}"/>
     <cellStyle name="Hyperlink 53" xfId="107" xr:uid="{00000000-0005-0000-0000-00007F010000}"/>
+    <cellStyle name="Hyperlink 54" xfId="236" hidden="1" xr:uid="{00000000-0005-0000-0000-000081010000}"/>
     <cellStyle name="Hyperlink 54" xfId="169" hidden="1" xr:uid="{00000000-0005-0000-0000-000080010000}"/>
-    <cellStyle name="Hyperlink 54" xfId="236" hidden="1" xr:uid="{00000000-0005-0000-0000-000081010000}"/>
     <cellStyle name="Hyperlink 54" xfId="108" xr:uid="{00000000-0005-0000-0000-000082010000}"/>
+    <cellStyle name="Hyperlink 55" xfId="235" hidden="1" xr:uid="{00000000-0005-0000-0000-000084010000}"/>
     <cellStyle name="Hyperlink 55" xfId="170" hidden="1" xr:uid="{00000000-0005-0000-0000-000083010000}"/>
-    <cellStyle name="Hyperlink 55" xfId="235" hidden="1" xr:uid="{00000000-0005-0000-0000-000084010000}"/>
     <cellStyle name="Hyperlink 55" xfId="109" xr:uid="{00000000-0005-0000-0000-000085010000}"/>
+    <cellStyle name="Hyperlink 56" xfId="234" hidden="1" xr:uid="{00000000-0005-0000-0000-000087010000}"/>
     <cellStyle name="Hyperlink 56" xfId="171" hidden="1" xr:uid="{00000000-0005-0000-0000-000086010000}"/>
-    <cellStyle name="Hyperlink 56" xfId="234" hidden="1" xr:uid="{00000000-0005-0000-0000-000087010000}"/>
     <cellStyle name="Hyperlink 56" xfId="110" xr:uid="{00000000-0005-0000-0000-000088010000}"/>
+    <cellStyle name="Hyperlink 57" xfId="233" hidden="1" xr:uid="{00000000-0005-0000-0000-00008A010000}"/>
     <cellStyle name="Hyperlink 57" xfId="172" hidden="1" xr:uid="{00000000-0005-0000-0000-000089010000}"/>
-    <cellStyle name="Hyperlink 57" xfId="233" hidden="1" xr:uid="{00000000-0005-0000-0000-00008A010000}"/>
     <cellStyle name="Hyperlink 57" xfId="111" xr:uid="{00000000-0005-0000-0000-00008B010000}"/>
+    <cellStyle name="Hyperlink 58" xfId="289" hidden="1" xr:uid="{00000000-0005-0000-0000-00008D010000}"/>
     <cellStyle name="Hyperlink 58" xfId="173" hidden="1" xr:uid="{00000000-0005-0000-0000-00008C010000}"/>
-    <cellStyle name="Hyperlink 58" xfId="289" hidden="1" xr:uid="{00000000-0005-0000-0000-00008D010000}"/>
     <cellStyle name="Hyperlink 58" xfId="624" xr:uid="{00000000-0005-0000-0000-00008E010000}"/>
+    <cellStyle name="Hyperlink 59" xfId="232" hidden="1" xr:uid="{00000000-0005-0000-0000-000090010000}"/>
     <cellStyle name="Hyperlink 59" xfId="174" hidden="1" xr:uid="{00000000-0005-0000-0000-00008F010000}"/>
-    <cellStyle name="Hyperlink 59" xfId="232" hidden="1" xr:uid="{00000000-0005-0000-0000-000090010000}"/>
     <cellStyle name="Hyperlink 59" xfId="112" xr:uid="{00000000-0005-0000-0000-000091010000}"/>
+    <cellStyle name="Hyperlink 6" xfId="284" hidden="1" xr:uid="{00000000-0005-0000-0000-000093010000}"/>
     <cellStyle name="Hyperlink 6" xfId="121" hidden="1" xr:uid="{00000000-0005-0000-0000-000092010000}"/>
-    <cellStyle name="Hyperlink 6" xfId="284" hidden="1" xr:uid="{00000000-0005-0000-0000-000093010000}"/>
     <cellStyle name="Hyperlink 6" xfId="619" xr:uid="{00000000-0005-0000-0000-000094010000}"/>
+    <cellStyle name="Hyperlink 60" xfId="290" hidden="1" xr:uid="{00000000-0005-0000-0000-000096010000}"/>
     <cellStyle name="Hyperlink 60" xfId="175" hidden="1" xr:uid="{00000000-0005-0000-0000-000095010000}"/>
-    <cellStyle name="Hyperlink 60" xfId="290" hidden="1" xr:uid="{00000000-0005-0000-0000-000096010000}"/>
     <cellStyle name="Hyperlink 60" xfId="625" xr:uid="{00000000-0005-0000-0000-000097010000}"/>
+    <cellStyle name="Hyperlink 61" xfId="291" hidden="1" xr:uid="{00000000-0005-0000-0000-000099010000}"/>
     <cellStyle name="Hyperlink 61" xfId="176" hidden="1" xr:uid="{00000000-0005-0000-0000-000098010000}"/>
-    <cellStyle name="Hyperlink 61" xfId="291" hidden="1" xr:uid="{00000000-0005-0000-0000-000099010000}"/>
     <cellStyle name="Hyperlink 61" xfId="626" xr:uid="{00000000-0005-0000-0000-00009A010000}"/>
+    <cellStyle name="Hyperlink 62" xfId="292" hidden="1" xr:uid="{00000000-0005-0000-0000-00009C010000}"/>
     <cellStyle name="Hyperlink 62" xfId="177" hidden="1" xr:uid="{00000000-0005-0000-0000-00009B010000}"/>
-    <cellStyle name="Hyperlink 62" xfId="292" hidden="1" xr:uid="{00000000-0005-0000-0000-00009C010000}"/>
     <cellStyle name="Hyperlink 62" xfId="627" xr:uid="{00000000-0005-0000-0000-00009D010000}"/>
+    <cellStyle name="Hyperlink 63" xfId="293" hidden="1" xr:uid="{00000000-0005-0000-0000-00009F010000}"/>
     <cellStyle name="Hyperlink 63" xfId="178" hidden="1" xr:uid="{00000000-0005-0000-0000-00009E010000}"/>
-    <cellStyle name="Hyperlink 63" xfId="293" hidden="1" xr:uid="{00000000-0005-0000-0000-00009F010000}"/>
     <cellStyle name="Hyperlink 63" xfId="628" xr:uid="{00000000-0005-0000-0000-0000A0010000}"/>
+    <cellStyle name="Hyperlink 64" xfId="294" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A2010000}"/>
     <cellStyle name="Hyperlink 64" xfId="179" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A1010000}"/>
-    <cellStyle name="Hyperlink 64" xfId="294" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A2010000}"/>
     <cellStyle name="Hyperlink 64" xfId="629" xr:uid="{00000000-0005-0000-0000-0000A3010000}"/>
+    <cellStyle name="Hyperlink 65" xfId="295" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A5010000}"/>
     <cellStyle name="Hyperlink 65" xfId="180" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A4010000}"/>
-    <cellStyle name="Hyperlink 65" xfId="295" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A5010000}"/>
     <cellStyle name="Hyperlink 65" xfId="630" xr:uid="{00000000-0005-0000-0000-0000A6010000}"/>
+    <cellStyle name="Hyperlink 66" xfId="296" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A8010000}"/>
     <cellStyle name="Hyperlink 66" xfId="181" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A7010000}"/>
-    <cellStyle name="Hyperlink 66" xfId="296" hidden="1" xr:uid="{00000000-0005-0000-0000-0000A8010000}"/>
     <cellStyle name="Hyperlink 66" xfId="631" xr:uid="{00000000-0005-0000-0000-0000A9010000}"/>
+    <cellStyle name="Hyperlink 67" xfId="297" hidden="1" xr:uid="{00000000-0005-0000-0000-0000AB010000}"/>
     <cellStyle name="Hyperlink 67" xfId="182" hidden="1" xr:uid="{00000000-0005-0000-0000-0000AA010000}"/>
-    <cellStyle name="Hyperlink 67" xfId="297" hidden="1" xr:uid="{00000000-0005-0000-0000-0000AB010000}"/>
     <cellStyle name="Hyperlink 67" xfId="632" xr:uid="{00000000-0005-0000-0000-0000AC010000}"/>
+    <cellStyle name="Hyperlink 68" xfId="298" hidden="1" xr:uid="{00000000-0005-0000-0000-0000AE010000}"/>
     <cellStyle name="Hyperlink 68" xfId="183" hidden="1" xr:uid="{00000000-0005-0000-0000-0000AD010000}"/>
-    <cellStyle name="Hyperlink 68" xfId="298" hidden="1" xr:uid="{00000000-0005-0000-0000-0000AE010000}"/>
     <cellStyle name="Hyperlink 68" xfId="633" xr:uid="{00000000-0005-0000-0000-0000AF010000}"/>
+    <cellStyle name="Hyperlink 69" xfId="299" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B1010000}"/>
     <cellStyle name="Hyperlink 69" xfId="184" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B0010000}"/>
-    <cellStyle name="Hyperlink 69" xfId="299" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B1010000}"/>
     <cellStyle name="Hyperlink 69" xfId="634" xr:uid="{00000000-0005-0000-0000-0000B2010000}"/>
+    <cellStyle name="Hyperlink 7" xfId="283" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B4010000}"/>
     <cellStyle name="Hyperlink 7" xfId="122" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B3010000}"/>
-    <cellStyle name="Hyperlink 7" xfId="283" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B4010000}"/>
     <cellStyle name="Hyperlink 7" xfId="618" xr:uid="{00000000-0005-0000-0000-0000B5010000}"/>
+    <cellStyle name="Hyperlink 70" xfId="300" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B7010000}"/>
     <cellStyle name="Hyperlink 70" xfId="185" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B6010000}"/>
-    <cellStyle name="Hyperlink 70" xfId="300" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B7010000}"/>
     <cellStyle name="Hyperlink 70" xfId="635" xr:uid="{00000000-0005-0000-0000-0000B8010000}"/>
+    <cellStyle name="Hyperlink 71" xfId="301" hidden="1" xr:uid="{00000000-0005-0000-0000-0000BA010000}"/>
     <cellStyle name="Hyperlink 71" xfId="186" hidden="1" xr:uid="{00000000-0005-0000-0000-0000B9010000}"/>
-    <cellStyle name="Hyperlink 71" xfId="301" hidden="1" xr:uid="{00000000-0005-0000-0000-0000BA010000}"/>
     <cellStyle name="Hyperlink 71" xfId="636" xr:uid="{00000000-0005-0000-0000-0000BB010000}"/>
+    <cellStyle name="Hyperlink 72" xfId="302" hidden="1" xr:uid="{00000000-0005-0000-0000-0000BD010000}"/>
     <cellStyle name="Hyperlink 72" xfId="187" hidden="1" xr:uid="{00000000-0005-0000-0000-0000BC010000}"/>
-    <cellStyle name="Hyperlink 72" xfId="302" hidden="1" xr:uid="{00000000-0005-0000-0000-0000BD010000}"/>
     <cellStyle name="Hyperlink 72" xfId="637" xr:uid="{00000000-0005-0000-0000-0000BE010000}"/>
+    <cellStyle name="Hyperlink 73" xfId="303" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C0010000}"/>
     <cellStyle name="Hyperlink 73" xfId="188" hidden="1" xr:uid="{00000000-0005-0000-0000-0000BF010000}"/>
-    <cellStyle name="Hyperlink 73" xfId="303" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C0010000}"/>
     <cellStyle name="Hyperlink 73" xfId="638" xr:uid="{00000000-0005-0000-0000-0000C1010000}"/>
+    <cellStyle name="Hyperlink 74" xfId="304" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C3010000}"/>
     <cellStyle name="Hyperlink 74" xfId="189" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C2010000}"/>
-    <cellStyle name="Hyperlink 74" xfId="304" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C3010000}"/>
     <cellStyle name="Hyperlink 74" xfId="639" xr:uid="{00000000-0005-0000-0000-0000C4010000}"/>
+    <cellStyle name="Hyperlink 75" xfId="305" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C6010000}"/>
     <cellStyle name="Hyperlink 75" xfId="190" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C5010000}"/>
-    <cellStyle name="Hyperlink 75" xfId="305" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C6010000}"/>
     <cellStyle name="Hyperlink 75" xfId="640" xr:uid="{00000000-0005-0000-0000-0000C7010000}"/>
+    <cellStyle name="Hyperlink 76" xfId="306" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C9010000}"/>
     <cellStyle name="Hyperlink 76" xfId="191" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C8010000}"/>
-    <cellStyle name="Hyperlink 76" xfId="306" hidden="1" xr:uid="{00000000-0005-0000-0000-0000C9010000}"/>
     <cellStyle name="Hyperlink 76" xfId="641" xr:uid="{00000000-0005-0000-0000-0000CA010000}"/>
+    <cellStyle name="Hyperlink 77" xfId="307" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CC010000}"/>
     <cellStyle name="Hyperlink 77" xfId="192" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CB010000}"/>
-    <cellStyle name="Hyperlink 77" xfId="307" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CC010000}"/>
     <cellStyle name="Hyperlink 77" xfId="642" xr:uid="{00000000-0005-0000-0000-0000CD010000}"/>
+    <cellStyle name="Hyperlink 78" xfId="308" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CF010000}"/>
     <cellStyle name="Hyperlink 78" xfId="193" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CE010000}"/>
-    <cellStyle name="Hyperlink 78" xfId="308" hidden="1" xr:uid="{00000000-0005-0000-0000-0000CF010000}"/>
     <cellStyle name="Hyperlink 78" xfId="643" xr:uid="{00000000-0005-0000-0000-0000D0010000}"/>
+    <cellStyle name="Hyperlink 79" xfId="309" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D2010000}"/>
     <cellStyle name="Hyperlink 79" xfId="194" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D1010000}"/>
-    <cellStyle name="Hyperlink 79" xfId="309" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D2010000}"/>
     <cellStyle name="Hyperlink 79" xfId="644" xr:uid="{00000000-0005-0000-0000-0000D3010000}"/>
+    <cellStyle name="Hyperlink 8" xfId="282" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D5010000}"/>
     <cellStyle name="Hyperlink 8" xfId="123" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D4010000}"/>
-    <cellStyle name="Hyperlink 8" xfId="282" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D5010000}"/>
     <cellStyle name="Hyperlink 8" xfId="617" xr:uid="{00000000-0005-0000-0000-0000D6010000}"/>
+    <cellStyle name="Hyperlink 80" xfId="310" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D8010000}"/>
     <cellStyle name="Hyperlink 80" xfId="195" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D7010000}"/>
-    <cellStyle name="Hyperlink 80" xfId="310" hidden="1" xr:uid="{00000000-0005-0000-0000-0000D8010000}"/>
     <cellStyle name="Hyperlink 80" xfId="645" xr:uid="{00000000-0005-0000-0000-0000D9010000}"/>
+    <cellStyle name="Hyperlink 81" xfId="311" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DB010000}"/>
     <cellStyle name="Hyperlink 81" xfId="196" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DA010000}"/>
-    <cellStyle name="Hyperlink 81" xfId="311" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DB010000}"/>
     <cellStyle name="Hyperlink 81" xfId="646" xr:uid="{00000000-0005-0000-0000-0000DC010000}"/>
+    <cellStyle name="Hyperlink 82" xfId="312" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DE010000}"/>
     <cellStyle name="Hyperlink 82" xfId="197" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DD010000}"/>
-    <cellStyle name="Hyperlink 82" xfId="312" hidden="1" xr:uid="{00000000-0005-0000-0000-0000DE010000}"/>
     <cellStyle name="Hyperlink 82" xfId="647" xr:uid="{00000000-0005-0000-0000-0000DF010000}"/>
+    <cellStyle name="Hyperlink 83" xfId="313" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E1010000}"/>
     <cellStyle name="Hyperlink 83" xfId="198" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E0010000}"/>
-    <cellStyle name="Hyperlink 83" xfId="313" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E1010000}"/>
     <cellStyle name="Hyperlink 83" xfId="648" xr:uid="{00000000-0005-0000-0000-0000E2010000}"/>
+    <cellStyle name="Hyperlink 84" xfId="314" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E4010000}"/>
     <cellStyle name="Hyperlink 84" xfId="199" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E3010000}"/>
-    <cellStyle name="Hyperlink 84" xfId="314" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E4010000}"/>
     <cellStyle name="Hyperlink 84" xfId="649" xr:uid="{00000000-0005-0000-0000-0000E5010000}"/>
+    <cellStyle name="Hyperlink 85" xfId="315" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E7010000}"/>
     <cellStyle name="Hyperlink 85" xfId="200" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E6010000}"/>
-    <cellStyle name="Hyperlink 85" xfId="315" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E7010000}"/>
     <cellStyle name="Hyperlink 85" xfId="650" xr:uid="{00000000-0005-0000-0000-0000E8010000}"/>
+    <cellStyle name="Hyperlink 86" xfId="316" hidden="1" xr:uid="{00000000-0005-0000-0000-0000EA010000}"/>
     <cellStyle name="Hyperlink 86" xfId="201" hidden="1" xr:uid="{00000000-0005-0000-0000-0000E9010000}"/>
-    <cellStyle name="Hyperlink 86" xfId="316" hidden="1" xr:uid="{00000000-0005-0000-0000-0000EA010000}"/>
     <cellStyle name="Hyperlink 86" xfId="651" xr:uid="{00000000-0005-0000-0000-0000EB010000}"/>
+    <cellStyle name="Hyperlink 87" xfId="317" hidden="1" xr:uid="{00000000-0005-0000-0000-0000ED010000}"/>
     <cellStyle name="Hyperlink 87" xfId="202" hidden="1" xr:uid="{00000000-0005-0000-0000-0000EC010000}"/>
-    <cellStyle name="Hyperlink 87" xfId="317" hidden="1" xr:uid="{00000000-0005-0000-0000-0000ED010000}"/>
     <cellStyle name="Hyperlink 87" xfId="652" xr:uid="{00000000-0005-0000-0000-0000EE010000}"/>
+    <cellStyle name="Hyperlink 88" xfId="318" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F0010000}"/>
     <cellStyle name="Hyperlink 88" xfId="203" hidden="1" xr:uid="{00000000-0005-0000-0000-0000EF010000}"/>
-    <cellStyle name="Hyperlink 88" xfId="318" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F0010000}"/>
     <cellStyle name="Hyperlink 88" xfId="653" xr:uid="{00000000-0005-0000-0000-0000F1010000}"/>
+    <cellStyle name="Hyperlink 89" xfId="319" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F3010000}"/>
     <cellStyle name="Hyperlink 89" xfId="204" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F2010000}"/>
-    <cellStyle name="Hyperlink 89" xfId="319" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F3010000}"/>
     <cellStyle name="Hyperlink 89" xfId="654" xr:uid="{00000000-0005-0000-0000-0000F4010000}"/>
+    <cellStyle name="Hyperlink 9" xfId="281" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F6010000}"/>
     <cellStyle name="Hyperlink 9" xfId="124" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F5010000}"/>
-    <cellStyle name="Hyperlink 9" xfId="281" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F6010000}"/>
     <cellStyle name="Hyperlink 9" xfId="616" xr:uid="{00000000-0005-0000-0000-0000F7010000}"/>
+    <cellStyle name="Hyperlink 90" xfId="320" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F9010000}"/>
     <cellStyle name="Hyperlink 90" xfId="205" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F8010000}"/>
-    <cellStyle name="Hyperlink 90" xfId="320" hidden="1" xr:uid="{00000000-0005-0000-0000-0000F9010000}"/>
     <cellStyle name="Hyperlink 90" xfId="655" xr:uid="{00000000-0005-0000-0000-0000FA010000}"/>
+    <cellStyle name="Hyperlink 91" xfId="321" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FC010000}"/>
     <cellStyle name="Hyperlink 91" xfId="206" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FB010000}"/>
-    <cellStyle name="Hyperlink 91" xfId="321" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FC010000}"/>
     <cellStyle name="Hyperlink 91" xfId="656" xr:uid="{00000000-0005-0000-0000-0000FD010000}"/>
+    <cellStyle name="Hyperlink 92" xfId="322" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FF010000}"/>
     <cellStyle name="Hyperlink 92" xfId="207" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FE010000}"/>
-    <cellStyle name="Hyperlink 92" xfId="322" hidden="1" xr:uid="{00000000-0005-0000-0000-0000FF010000}"/>
     <cellStyle name="Hyperlink 92" xfId="657" xr:uid="{00000000-0005-0000-0000-000000020000}"/>
+    <cellStyle name="Hyperlink 93" xfId="323" hidden="1" xr:uid="{00000000-0005-0000-0000-000002020000}"/>
     <cellStyle name="Hyperlink 93" xfId="208" hidden="1" xr:uid="{00000000-0005-0000-0000-000001020000}"/>
-    <cellStyle name="Hyperlink 93" xfId="323" hidden="1" xr:uid="{00000000-0005-0000-0000-000002020000}"/>
     <cellStyle name="Hyperlink 93" xfId="658" xr:uid="{00000000-0005-0000-0000-000003020000}"/>
+    <cellStyle name="Hyperlink 94" xfId="324" hidden="1" xr:uid="{00000000-0005-0000-0000-000005020000}"/>
     <cellStyle name="Hyperlink 94" xfId="209" hidden="1" xr:uid="{00000000-0005-0000-0000-000004020000}"/>
-    <cellStyle name="Hyperlink 94" xfId="324" hidden="1" xr:uid="{00000000-0005-0000-0000-000005020000}"/>
     <cellStyle name="Hyperlink 94" xfId="659" xr:uid="{00000000-0005-0000-0000-000006020000}"/>
+    <cellStyle name="Hyperlink 95" xfId="325" hidden="1" xr:uid="{00000000-0005-0000-0000-000008020000}"/>
     <cellStyle name="Hyperlink 95" xfId="210" hidden="1" xr:uid="{00000000-0005-0000-0000-000007020000}"/>
-    <cellStyle name="Hyperlink 95" xfId="325" hidden="1" xr:uid="{00000000-0005-0000-0000-000008020000}"/>
     <cellStyle name="Hyperlink 95" xfId="660" xr:uid="{00000000-0005-0000-0000-000009020000}"/>
+    <cellStyle name="Hyperlink 96" xfId="326" hidden="1" xr:uid="{00000000-0005-0000-0000-00000B020000}"/>
     <cellStyle name="Hyperlink 96" xfId="211" hidden="1" xr:uid="{00000000-0005-0000-0000-00000A020000}"/>
-    <cellStyle name="Hyperlink 96" xfId="326" hidden="1" xr:uid="{00000000-0005-0000-0000-00000B020000}"/>
     <cellStyle name="Hyperlink 96" xfId="661" xr:uid="{00000000-0005-0000-0000-00000C020000}"/>
+    <cellStyle name="Hyperlink 97" xfId="327" hidden="1" xr:uid="{00000000-0005-0000-0000-00000E020000}"/>
     <cellStyle name="Hyperlink 97" xfId="212" hidden="1" xr:uid="{00000000-0005-0000-0000-00000D020000}"/>
-    <cellStyle name="Hyperlink 97" xfId="327" hidden="1" xr:uid="{00000000-0005-0000-0000-00000E020000}"/>
     <cellStyle name="Hyperlink 97" xfId="662" xr:uid="{00000000-0005-0000-0000-00000F020000}"/>
+    <cellStyle name="Hyperlink 98" xfId="328" hidden="1" xr:uid="{00000000-0005-0000-0000-000011020000}"/>
     <cellStyle name="Hyperlink 98" xfId="213" hidden="1" xr:uid="{00000000-0005-0000-0000-000010020000}"/>
-    <cellStyle name="Hyperlink 98" xfId="328" hidden="1" xr:uid="{00000000-0005-0000-0000-000011020000}"/>
     <cellStyle name="Hyperlink 98" xfId="663" xr:uid="{00000000-0005-0000-0000-000012020000}"/>
+    <cellStyle name="Hyperlink 99" xfId="329" hidden="1" xr:uid="{00000000-0005-0000-0000-000014020000}"/>
     <cellStyle name="Hyperlink 99" xfId="214" hidden="1" xr:uid="{00000000-0005-0000-0000-000013020000}"/>
-    <cellStyle name="Hyperlink 99" xfId="329" hidden="1" xr:uid="{00000000-0005-0000-0000-000014020000}"/>
     <cellStyle name="Hyperlink 99" xfId="664" xr:uid="{00000000-0005-0000-0000-000015020000}"/>
     <cellStyle name="Input" xfId="23" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Input [yellow]" xfId="481" xr:uid="{00000000-0005-0000-0000-000017020000}"/>
@@ -4171,9 +4174,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="132.28515625" customWidth="1"/>
+    <col min="2" max="2" width="132.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -4205,7 +4208,7 @@
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="B7" s="62" t="s">
+      <c r="B7" s="61" t="s">
         <v>5</v>
       </c>
     </row>
@@ -4264,15 +4267,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:X44"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.140625" customWidth="1"/>
-    <col min="13" max="13" width="18.140625" customWidth="1"/>
-    <col min="18" max="18" width="14.7109375" customWidth="1"/>
-    <col min="19" max="19" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.109375" customWidth="1"/>
+    <col min="13" max="13" width="18.109375" customWidth="1"/>
+    <col min="18" max="18" width="14.6640625" customWidth="1"/>
+    <col min="19" max="19" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24">
@@ -4293,10 +4296,10 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
-      <c r="M2" s="31" t="s">
+      <c r="M2" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="31" t="s">
+      <c r="N2" s="30" t="s">
         <v>18</v>
       </c>
       <c r="Q2" s="2" t="s">
@@ -4306,19 +4309,19 @@
       <c r="S2" s="6"/>
     </row>
     <row r="3" spans="1:24">
-      <c r="A3" s="32">
+      <c r="A3" s="31">
         <v>7.3</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="34" t="s">
+      <c r="B3" s="32"/>
+      <c r="C3" s="33" t="s">
         <v>19</v>
       </c>
       <c r="D3" s="19"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
       <c r="M3" s="24" t="s">
         <v>20</v>
       </c>
@@ -4327,25 +4330,25 @@
         <v>6.3</v>
       </c>
       <c r="Q3" s="18"/>
-      <c r="R3" s="34" t="s">
+      <c r="R3" s="33" t="s">
         <v>19</v>
       </c>
       <c r="S3" s="19"/>
       <c r="T3" s="19"/>
-      <c r="U3" s="36"/>
-      <c r="V3" s="36"/>
-      <c r="W3" s="36"/>
+      <c r="U3" s="35"/>
+      <c r="V3" s="35"/>
+      <c r="W3" s="35"/>
     </row>
     <row r="4" spans="1:24">
-      <c r="A4" s="32"/>
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
+      <c r="A4" s="31"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="33"/>
       <c r="D4" s="19"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
       <c r="M4" s="22" t="s">
         <v>21</v>
       </c>
@@ -4354,31 +4357,31 @@
       <c r="R4" s="19"/>
       <c r="S4" s="19"/>
       <c r="T4" s="19"/>
-      <c r="U4" s="36"/>
-      <c r="V4" s="36"/>
-      <c r="W4" s="36"/>
+      <c r="U4" s="35"/>
+      <c r="V4" s="35"/>
+      <c r="W4" s="35"/>
     </row>
     <row r="5" spans="1:24">
-      <c r="A5" s="32"/>
-      <c r="B5" s="33"/>
-      <c r="C5" s="37" t="s">
+      <c r="A5" s="31"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="37" t="s">
+      <c r="E5" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="37" t="s">
+      <c r="F5" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38">
+      <c r="G5" s="36"/>
+      <c r="H5" s="37">
         <f>base.year</f>
         <v>2020</v>
       </c>
-      <c r="I5" s="38">
+      <c r="I5" s="37">
         <v>2022</v>
       </c>
       <c r="J5" s="1">
@@ -4392,21 +4395,21 @@
       </c>
       <c r="N5" s="22"/>
       <c r="Q5" s="18"/>
-      <c r="R5" s="54" t="s">
+      <c r="R5" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="S5" s="54" t="s">
+      <c r="S5" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="T5" s="54" t="s">
+      <c r="T5" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="U5" s="55"/>
-      <c r="V5" s="38">
+      <c r="U5" s="54"/>
+      <c r="V5" s="37">
         <f>base.year</f>
         <v>2020</v>
       </c>
-      <c r="W5" s="38">
+      <c r="W5" s="37">
         <v>2022</v>
       </c>
       <c r="X5" s="1">
@@ -4414,23 +4417,23 @@
       </c>
     </row>
     <row r="6" spans="1:24">
-      <c r="A6" s="32"/>
-      <c r="B6" s="33"/>
-      <c r="C6" s="39" t="s">
+      <c r="A6" s="31"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="40" t="s">
+      <c r="E6" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="41">
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="40">
         <v>10</v>
       </c>
-      <c r="I6" s="42">
+      <c r="I6" s="41">
         <v>10</v>
       </c>
       <c r="J6" s="9">
@@ -4453,11 +4456,11 @@
       <c r="T6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="U6" s="36"/>
-      <c r="V6" s="36">
+      <c r="U6" s="35"/>
+      <c r="V6" s="35">
         <v>10</v>
       </c>
-      <c r="W6" s="36">
+      <c r="W6" s="35">
         <v>10</v>
       </c>
       <c r="X6">
@@ -4466,19 +4469,19 @@
       </c>
     </row>
     <row r="7" spans="1:24">
-      <c r="A7" s="32"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="40" t="s">
+      <c r="A7" s="31"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="40"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="41">
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="40">
         <v>10</v>
       </c>
-      <c r="I7" s="42">
+      <c r="I7" s="41">
         <v>10</v>
       </c>
       <c r="J7" s="9">
@@ -4498,11 +4501,11 @@
       <c r="T7" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="U7" s="36"/>
-      <c r="V7" s="36">
+      <c r="U7" s="35"/>
+      <c r="V7" s="35">
         <v>10</v>
       </c>
-      <c r="W7" s="36">
+      <c r="W7" s="35">
         <v>10</v>
       </c>
       <c r="X7">
@@ -4511,19 +4514,19 @@
       </c>
     </row>
     <row r="8" spans="1:24">
-      <c r="A8" s="32"/>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="40" t="s">
+      <c r="A8" s="31"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="41">
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40">
         <v>10</v>
       </c>
-      <c r="I8" s="42">
+      <c r="I8" s="41">
         <v>10</v>
       </c>
       <c r="J8" s="9">
@@ -4542,11 +4545,11 @@
       <c r="T8" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="U8" s="36"/>
-      <c r="V8" s="36">
+      <c r="U8" s="35"/>
+      <c r="V8" s="35">
         <v>10</v>
       </c>
-      <c r="W8" s="36">
+      <c r="W8" s="35">
         <v>10</v>
       </c>
       <c r="X8">
@@ -4555,19 +4558,19 @@
       </c>
     </row>
     <row r="9" spans="1:24">
-      <c r="A9" s="32"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="40" t="s">
+      <c r="A9" s="31"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="41">
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="40">
         <v>10</v>
       </c>
-      <c r="I9" s="42">
+      <c r="I9" s="41">
         <v>10</v>
       </c>
       <c r="J9" s="9">
@@ -4592,11 +4595,11 @@
       <c r="T9" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="U9" s="36"/>
-      <c r="V9" s="36">
+      <c r="U9" s="35"/>
+      <c r="V9" s="35">
         <v>10</v>
       </c>
-      <c r="W9" s="36">
+      <c r="W9" s="35">
         <v>10</v>
       </c>
       <c r="X9">
@@ -4605,21 +4608,21 @@
       </c>
     </row>
     <row r="10" spans="1:24">
-      <c r="A10" s="32"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="39" t="s">
+      <c r="A10" s="31"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="40" t="s">
+      <c r="E10" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="41">
+      <c r="F10" s="39"/>
+      <c r="G10" s="39"/>
+      <c r="H10" s="40">
         <v>10</v>
       </c>
-      <c r="I10" s="42">
+      <c r="I10" s="41">
         <v>10</v>
       </c>
       <c r="J10" s="9">
@@ -4633,14 +4636,14 @@
       <c r="Q10" s="18"/>
       <c r="R10" s="19"/>
       <c r="S10" s="19"/>
-      <c r="T10" s="40" t="s">
+      <c r="T10" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="U10" s="36"/>
-      <c r="V10" s="36">
+      <c r="U10" s="35"/>
+      <c r="V10" s="35">
         <v>10</v>
       </c>
-      <c r="W10" s="36">
+      <c r="W10" s="35">
         <v>10</v>
       </c>
       <c r="X10">
@@ -4649,19 +4652,19 @@
       </c>
     </row>
     <row r="11" spans="1:24">
-      <c r="A11" s="32"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="40" t="s">
+      <c r="A11" s="31"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="41">
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="40">
         <v>10</v>
       </c>
-      <c r="I11" s="42">
+      <c r="I11" s="41">
         <v>10</v>
       </c>
       <c r="J11" s="9">
@@ -4680,11 +4683,11 @@
       <c r="T11" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="U11" s="36"/>
-      <c r="V11" s="36">
+      <c r="U11" s="35"/>
+      <c r="V11" s="35">
         <v>10</v>
       </c>
-      <c r="W11" s="36">
+      <c r="W11" s="35">
         <v>10</v>
       </c>
       <c r="X11">
@@ -4693,21 +4696,21 @@
       </c>
     </row>
     <row r="12" spans="1:24">
-      <c r="A12" s="32"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="39" t="s">
+      <c r="A12" s="31"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="40" t="s">
+      <c r="E12" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="41">
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="40">
         <v>20</v>
       </c>
-      <c r="I12" s="42">
+      <c r="I12" s="41">
         <v>20</v>
       </c>
       <c r="J12" s="9">
@@ -4728,11 +4731,11 @@
       <c r="T12" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="U12" s="36"/>
-      <c r="V12" s="36">
+      <c r="U12" s="35"/>
+      <c r="V12" s="35">
         <v>35</v>
       </c>
-      <c r="W12" s="36">
+      <c r="W12" s="35">
         <v>35</v>
       </c>
       <c r="X12">
@@ -4741,19 +4744,19 @@
       </c>
     </row>
     <row r="13" spans="1:24">
-      <c r="A13" s="32"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="33"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="40" t="s">
+      <c r="A13" s="31"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="40"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="41">
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="40">
         <v>20</v>
       </c>
-      <c r="I13" s="42">
+      <c r="I13" s="41">
         <v>20</v>
       </c>
       <c r="J13" s="9">
@@ -4772,11 +4775,11 @@
       <c r="T13" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="U13" s="36"/>
-      <c r="V13" s="36">
+      <c r="U13" s="35"/>
+      <c r="V13" s="35">
         <v>35</v>
       </c>
-      <c r="W13" s="36">
+      <c r="W13" s="35">
         <v>35</v>
       </c>
       <c r="X13">
@@ -4785,19 +4788,19 @@
       </c>
     </row>
     <row r="14" spans="1:24">
-      <c r="A14" s="32"/>
-      <c r="B14" s="33"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="40" t="s">
+      <c r="A14" s="31"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
-      <c r="H14" s="41">
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="40">
         <v>15</v>
       </c>
-      <c r="I14" s="42">
+      <c r="I14" s="41">
         <v>15</v>
       </c>
       <c r="J14" s="9">
@@ -4818,11 +4821,11 @@
       <c r="T14" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="U14" s="36"/>
-      <c r="V14" s="56">
+      <c r="U14" s="35"/>
+      <c r="V14" s="55">
         <v>30</v>
       </c>
-      <c r="W14" s="56">
+      <c r="W14" s="55">
         <v>30</v>
       </c>
       <c r="X14">
@@ -4831,19 +4834,19 @@
       </c>
     </row>
     <row r="15" spans="1:24" ht="15.6">
-      <c r="A15" s="32"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="40" t="s">
+      <c r="A15" s="31"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="41">
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="40">
         <v>15</v>
       </c>
-      <c r="I15" s="42">
+      <c r="I15" s="41">
         <v>15</v>
       </c>
       <c r="J15" s="9">
@@ -4856,33 +4859,33 @@
         <v>10</v>
       </c>
       <c r="N15" s="22"/>
-      <c r="P15" s="57"/>
-      <c r="Q15" s="47"/>
-      <c r="R15" s="39" t="s">
+      <c r="P15" s="56"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="S15" s="39"/>
-      <c r="T15" s="40" t="s">
+      <c r="S15" s="38"/>
+      <c r="T15" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="U15" s="58"/>
-      <c r="V15" s="59"/>
-      <c r="W15" s="59"/>
+      <c r="U15" s="57"/>
+      <c r="V15" s="58"/>
+      <c r="W15" s="58"/>
     </row>
     <row r="16" spans="1:24" ht="15.6">
-      <c r="A16" s="32"/>
-      <c r="B16" s="33"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="44" t="s">
+      <c r="A16" s="31"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="F16" s="44"/>
-      <c r="G16" s="44"/>
-      <c r="H16" s="41">
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="40">
         <v>20</v>
       </c>
-      <c r="I16" s="42">
+      <c r="I16" s="41">
         <v>20</v>
       </c>
       <c r="J16" s="9">
@@ -4895,33 +4898,33 @@
         <v>50</v>
       </c>
       <c r="N16" s="22"/>
-      <c r="P16" s="57"/>
-      <c r="Q16" s="47"/>
-      <c r="R16" s="50"/>
-      <c r="S16" s="50"/>
-      <c r="T16" s="51" t="s">
+      <c r="P16" s="56"/>
+      <c r="Q16" s="46"/>
+      <c r="R16" s="49"/>
+      <c r="S16" s="49"/>
+      <c r="T16" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="U16" s="60"/>
-      <c r="V16" s="61"/>
-      <c r="W16" s="61"/>
+      <c r="U16" s="59"/>
+      <c r="V16" s="60"/>
+      <c r="W16" s="60"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="32"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="39" t="s">
+      <c r="A17" s="31"/>
+      <c r="B17" s="32"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="40" t="s">
+      <c r="E17" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="F17" s="40"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="41">
+      <c r="F17" s="39"/>
+      <c r="G17" s="39"/>
+      <c r="H17" s="40">
         <v>12</v>
       </c>
-      <c r="I17" s="42">
+      <c r="I17" s="41">
         <v>12</v>
       </c>
       <c r="J17" s="9">
@@ -4940,19 +4943,19 @@
       </c>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="32"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="40" t="s">
+      <c r="A18" s="31"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="41">
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="40">
         <v>12</v>
       </c>
-      <c r="I18" s="42">
+      <c r="I18" s="41">
         <v>12</v>
       </c>
       <c r="J18" s="9">
@@ -4965,21 +4968,21 @@
       <c r="N18" s="23"/>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="32"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="39" t="s">
+      <c r="A19" s="31"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="40" t="s">
+      <c r="E19" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="40"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="41">
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="40">
         <v>8</v>
       </c>
-      <c r="I19" s="42">
+      <c r="I19" s="41">
         <v>8</v>
       </c>
       <c r="J19" s="9">
@@ -4994,19 +4997,19 @@
       <c r="N19" s="27"/>
     </row>
     <row r="20" spans="1:14">
-      <c r="A20" s="32"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="33"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="40" t="s">
+      <c r="A20" s="31"/>
+      <c r="B20" s="32"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="41">
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="40">
         <v>8</v>
       </c>
-      <c r="I20" s="42">
+      <c r="I20" s="41">
         <v>8</v>
       </c>
       <c r="J20" s="9">
@@ -5021,19 +5024,19 @@
       <c r="N20" s="22"/>
     </row>
     <row r="21" spans="1:14">
-      <c r="A21" s="32"/>
-      <c r="B21" s="33"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="40" t="s">
+      <c r="A21" s="31"/>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="41">
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40">
         <v>5</v>
       </c>
-      <c r="I21" s="42">
+      <c r="I21" s="41">
         <v>5</v>
       </c>
       <c r="J21" s="9">
@@ -5050,21 +5053,21 @@
       </c>
     </row>
     <row r="22" spans="1:14">
-      <c r="A22" s="32"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="39" t="s">
+      <c r="A22" s="31"/>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="E22" s="40" t="s">
+      <c r="E22" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="41">
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="40">
         <v>8</v>
       </c>
-      <c r="I22" s="42">
+      <c r="I22" s="41">
         <v>8</v>
       </c>
       <c r="J22" s="9">
@@ -5077,19 +5080,19 @@
       <c r="N22" s="23"/>
     </row>
     <row r="23" spans="1:14">
-      <c r="A23" s="32"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40" t="s">
+      <c r="A23" s="31"/>
+      <c r="B23" s="32"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="45">
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="44">
         <v>8</v>
       </c>
-      <c r="I23" s="46">
+      <c r="I23" s="45">
         <v>8</v>
       </c>
       <c r="J23" s="9">
@@ -5104,19 +5107,19 @@
       <c r="N23" s="27"/>
     </row>
     <row r="24" spans="1:14">
-      <c r="A24" s="32"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="40" t="s">
+      <c r="A24" s="31"/>
+      <c r="B24" s="32"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="40"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="45">
+      <c r="F24" s="39"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="44">
         <v>12</v>
       </c>
-      <c r="I24" s="46">
+      <c r="I24" s="45">
         <v>12</v>
       </c>
       <c r="J24" s="9">
@@ -5131,23 +5134,23 @@
       <c r="N24" s="22"/>
     </row>
     <row r="25" spans="1:14">
-      <c r="A25" s="32"/>
-      <c r="B25" s="33"/>
-      <c r="C25" s="39" t="s">
+      <c r="A25" s="31"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="D25" s="39" t="s">
+      <c r="D25" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E25" s="40" t="s">
+      <c r="E25" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="41">
+      <c r="F25" s="39"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="40">
         <v>35</v>
       </c>
-      <c r="I25" s="42">
+      <c r="I25" s="41">
         <v>35</v>
       </c>
       <c r="J25" s="9">
@@ -5164,19 +5167,19 @@
       </c>
     </row>
     <row r="26" spans="1:14">
-      <c r="A26" s="32"/>
-      <c r="B26" s="33"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="40" t="s">
+      <c r="A26" s="31"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="F26" s="40"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="41">
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="40">
         <v>35</v>
       </c>
-      <c r="I26" s="42">
+      <c r="I26" s="41">
         <v>35</v>
       </c>
       <c r="J26" s="9">
@@ -5189,23 +5192,23 @@
       <c r="N26" s="23"/>
     </row>
     <row r="27" spans="1:14">
-      <c r="A27" s="32"/>
-      <c r="B27" s="33"/>
-      <c r="C27" s="39" t="s">
+      <c r="A27" s="31"/>
+      <c r="B27" s="32"/>
+      <c r="C27" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="D27" s="39" t="s">
+      <c r="D27" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="39" t="s">
+      <c r="E27" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="41">
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="40">
         <v>30</v>
       </c>
-      <c r="I27" s="41">
+      <c r="I27" s="40">
         <v>30</v>
       </c>
       <c r="J27" s="9">
@@ -5220,35 +5223,35 @@
       <c r="N27" s="2"/>
     </row>
     <row r="28" spans="1:14" ht="15.6">
-      <c r="A28" s="32"/>
-      <c r="B28" s="47"/>
-      <c r="C28" s="39" t="s">
+      <c r="A28" s="31"/>
+      <c r="B28" s="46"/>
+      <c r="C28" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="39"/>
-      <c r="E28" s="40" t="s">
+      <c r="D28" s="38"/>
+      <c r="E28" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="F28" s="48"/>
-      <c r="G28" s="48"/>
-      <c r="H28" s="49"/>
-      <c r="I28" s="49"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="47"/>
+      <c r="H28" s="48"/>
+      <c r="I28" s="48"/>
       <c r="M28" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="15.6">
-      <c r="A29" s="32"/>
-      <c r="B29" s="47"/>
-      <c r="C29" s="50"/>
-      <c r="D29" s="50"/>
-      <c r="E29" s="51" t="s">
+      <c r="A29" s="31"/>
+      <c r="B29" s="46"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="F29" s="52"/>
-      <c r="G29" s="52"/>
-      <c r="H29" s="53"/>
-      <c r="I29" s="53"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="51"/>
+      <c r="H29" s="52"/>
+      <c r="I29" s="52"/>
       <c r="M29" s="9">
         <f>AVERAGE(J17:J18)</f>
         <v>12</v>
@@ -5610,15 +5613,15 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="29.1">
+    <row r="1" spans="1:4" ht="28.8">
       <c r="A1" s="20" t="s">
         <v>66</v>
       </c>
@@ -5629,7 +5632,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
@@ -5642,7 +5645,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -5655,7 +5658,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -5668,7 +5671,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -5681,21 +5684,23 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="7">
-        <f>'India Data'!M7</f>
-        <v>9.3333333333333339</v>
-      </c>
-      <c r="C6" s="30">
+      <c r="B6" s="62">
         <v>33</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="C6" s="62">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B7" s="7">
         <f>'India Data'!M33</f>
@@ -5727,8 +5732,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A251C7805F896F47A4F48569C73A0799" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="378e06851fdbb175a3d0a15b25cca813">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f3083de3-5d4e-49f2-a3cd-0aeb079e6739" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1ff5ef3c1d0a8a18c2d988b302a3fc15" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A251C7805F896F47A4F48569C73A0799" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7abd873f26c83d98889b6bc5171c7cdd">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f3083de3-5d4e-49f2-a3cd-0aeb079e6739" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="295384f30983e71c631053ca9b14fb23" ns2:_="">
     <xsd:import namespace="f3083de3-5d4e-49f2-a3cd-0aeb079e6739"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -5739,6 +5744,7 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -5762,6 +5768,11 @@
     <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="11" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -5865,13 +5876,42 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0412D13-3EB8-4B19-AF90-A24E2BF3ED51}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0412D13-3EB8-4B19-AF90-A24E2BF3ED51}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2376E651-6287-4D79-AFC1-7510C33DB521}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2376E651-6287-4D79-AFC1-7510C33DB521}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D9380B6-8954-4B9A-8A48-E4D3B0D86AE0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BA23818-7B94-45EF-9F46-0D9A05135992}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f3083de3-5d4e-49f2-a3cd-0aeb079e6739"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{c7ef1c8b-ba63-4702-8e74-5094387a97de}" enabled="0" method="" siteId="{c7ef1c8b-ba63-4702-8e74-5094387a97de}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>